<commit_message>
feat(kebiasaan-baik): sumber rujukan untuk 77 kebiasaan, bisa diklik orang tua
- 29 rujukan terverifikasi (AAP/HealthyChildren, CDC, Harvard Center on the Developing Child,
  ZERO TO THREE, CFPB, dan riset ditelaah sejawat dengan DOI/PubMed) dipetakan ke setiap butir
- Migrasi 029: kolom kebiasaan_baik.sumber, isi awal untuk butir yang masih kosong,
  terapkan_kebiasaan ikut menyimpan sumber
- Tampil sebagai tautan ringkas di kartu kegiatan Irama Hari, Kebiasaan situasional (Kelola),
  dan daftar sikap di Bekal; data lama tanpa sumber memakai rujukan bawaan per ID
- Admin: kolom Sumber di editor (dengan pratinjau tautan), import/ekspor CSV & template Excel,
  perbandingan revisi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Czkp7HnUTKUNKpexU1deSc
</commit_message>
<xml_diff>
--- a/apps/digital/public/templates/Rekah_Template_Import_Kebiasaan_v1.xlsx
+++ b/apps/digital/public/templates/Rekah_Template_Import_Kebiasaan_v1.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,6 +497,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>urutan</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>sumber</t>
         </is>
       </c>
     </row>
@@ -518,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -531,9 +537,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -587,6 +591,13 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>7. Kegiatan template (nama, jam, urutan) diatur langsung di tab “Kegiatan template”, bukan lewat file ini.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8. sumber: rujukan (opsional), beberapa sumber dipisah titik koma (;). Tulis alamat web atau DOI agar tautan langsung ke halaman yang tepat.</t>
         </is>
       </c>
     </row>
@@ -601,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -614,6 +625,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,9 +679,13 @@
           <t>urutan</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>sumber</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>Pakai sandal sendiri sebelum keluar</t>
@@ -701,13 +717,16 @@
           <t>mandipagi</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>200</v>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Tepper dkk. (2022). Executive functions and household chores. https://doi.org/10.1111/1440-1630.12822</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>Tarik napas bersama</t>
@@ -734,7 +753,6 @@
           <t>situasional</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>saat anak kesal</t>
@@ -743,6 +761,11 @@
       <c r="J3" t="n">
         <v>200</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ZERO TO THREE — How to Help Children Develop Self-Control. https://www.zerotothree.org/resource/help-your-child-develop-self-control/</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -781,9 +804,13 @@
           <t>beres</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
         <v>129</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Tepper dkk. (2022). Executive functions and household chores. https://doi.org/10.1111/1440-1630.12822</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -866,13 +893,11 @@
           <t>Bangun tidur</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>Kejujuran</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>0–3 bl</t>
@@ -901,13 +926,11 @@
           <t>Sarapan</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>Syukur</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>3–6 bl</t>
@@ -936,13 +959,11 @@
           <t>Mandi pagi</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>Kasih Sayang</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>6–9 bl</t>
@@ -971,13 +992,11 @@
           <t>Main bersama</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Empati</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>9–12 bl</t>
@@ -1006,13 +1025,11 @@
           <t>Makan siang</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Kemandirian</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>12–18 bl</t>
@@ -1041,13 +1058,11 @@
           <t>Tidur siang</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Tanggung Jawab</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>18–24 bl</t>
@@ -1076,13 +1091,11 @@
           <t>Makan malam</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>Kesederhanaan</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2–3 th</t>
@@ -1111,13 +1124,11 @@
           <t>Beres-beres</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Cinta Ilmu</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>3–4 th</t>
@@ -1146,13 +1157,11 @@
           <t>Rutinitas sebelum tidur</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Sabar</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>4–5 th</t>
@@ -1166,16 +1175,11 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Berbagi</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>5–6 th</t>
@@ -1189,16 +1193,11 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Keberanian</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>Semua usia</t>
@@ -1212,19 +1211,11 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Hormat pada Sesama</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">

</xml_diff>